<commit_message>
Add safe print margins and update published status
</commit_message>
<xml_diff>
--- a/outputs/019feff7-57dd-78c0-aa99-aea2103fbc23-mail-response-20260926/紹介状機能_メール項目別対応一覧_20260926.xlsx
+++ b/outputs/019feff7-57dd-78c0-aa99-aea2103fbc23-mail-response-20260926/紹介状機能_メール項目別対応一覧_20260926.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール項目別対応表" sheetId="1" r:id="R5226a580ec83400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール項目別対応表" sheetId="1" r:id="Rf13cde9ccbc14948"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,20 +354,23 @@
     <x:row r="2" ht="97.5" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>全体
-2026年9月26日時点</x:v>
+2026年9月26日
+公開状況を更新</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
         <x:v>対象メール：9月25日23:45のご回答（件名「Re: 【トヨタ財団】調査票＆紹介状の実装について」）。以前の合意事項も併記。</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>下記の追加改修を実装し、開発環境で動作を確認しました。</x:v>
+        <x:v>今回の追加改修は先方確認用サイトへ反映済みです。最新コミット d149591 の公開処理成功と、公開画面で7問から紹介状作成までの操作を確認しました。
+確認先：https://feat-referral-letter.openfisca-japan.pages.dev/referral-letter</x:v>
       </x:c>
       <x:c r="D2" s="10" t="str">
-        <x:v>開発環境で確認済み
-自動テスト42件すべて成功。アプリのビルド・コードチェックも成功。</x:v>
+        <x:v>先方確認用サイトで確認済み
+更新後の相談先・電話案内・見出し・注意書きと、紹介状の相談先／バッジ非表示を確認。
+開発環境での全42件の自動テスト・ビルド等の成功結果も維持。</x:v>
       </x:c>
       <x:c r="E2" s="10" t="str">
-        <x:v>本表の「確認済み」は開発環境での結果です。今回の追加改修は公開サイトへの反映前です。実際の印刷時の改ページ確認は残っています。</x:v>
+        <x:v>各項目の全件照合・保存画像等は開発環境での確認結果です。公開サイトでは代表例を確認しました。実際の印刷時の改ページ確認は残っています。一般向け本番サイトへの反映とは別です。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="82.5" customHeight="1">
@@ -642,7 +645,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1820fac96b2e4376"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd428d2959cb74f4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add print margins and update referral letter review
</commit_message>
<xml_diff>
--- a/outputs/019feff7-57dd-78c0-aa99-aea2103fbc23-mail-response-20260926/紹介状機能_メール項目別対応一覧_20260926.xlsx
+++ b/outputs/019feff7-57dd-78c0-aa99-aea2103fbc23-mail-response-20260926/紹介状機能_メール項目別対応一覧_20260926.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール項目別対応表" sheetId="1" r:id="Rf13cde9ccbc14948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="メール項目別対応表" sheetId="1" r:id="R93bccfa4f0544708"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,8 +119,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MailResponse" displayName="MailResponse" ref="A1:E16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:E16"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MailResponse" displayName="MailResponse" ref="A1:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:E17"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="メールの該当項目"/>
     <x:tableColumn id="2" name="ご依頼・ご回答の要旨"/>
@@ -355,22 +355,21 @@
       <x:c r="A2" s="6" t="str">
         <x:v>全体
 2026年9月26日
-公開状況を更新</x:v>
+印刷確認結果を更新</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
         <x:v>対象メール：9月25日23:45のご回答（件名「Re: 【トヨタ財団】調査票＆紹介状の実装について」）。以前の合意事項も併記。</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>今回の追加改修は先方確認用サイトへ反映済みです。最新コミット d149591 の公開処理成功と、公開画面で7問から紹介状作成までの操作を確認しました。
+        <x:v>追加改修（d149591）は先方確認用サイトへ反映・代表操作確認済みです。その後、印刷時の左右10mmの余白を追加しました。
 確認先：https://feat-referral-letter.openfisca-japan.pages.dev/referral-letter</x:v>
       </x:c>
       <x:c r="D2" s="10" t="str">
-        <x:v>先方確認用サイトで確認済み
-更新後の相談先・電話案内・見出し・注意書きと、紹介状の相談先／バッジ非表示を確認。
-開発環境での全42件の自動テスト・ビルド等の成功結果も維持。</x:v>
+        <x:v>添付PDFでA4縦1ページの表示を確認済み。余白修正後の依存パッケージのインストール・ビルドも成功。
+全42件の自動テスト成功は余白修正前の結果です。</x:v>
       </x:c>
       <x:c r="E2" s="10" t="str">
-        <x:v>各項目の全件照合・保存画像等は開発環境での確認結果です。公開サイトでは代表例を確認しました。実際の印刷時の改ページ確認は残っています。一般向け本番サイトへの反映とは別です。</x:v>
+        <x:v>残る確認：余白修正後の公開反映・PDF再出力、複数ページになる場合の改ページ、実機印刷。一般向け本番サイトへの反映とは別です。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="82.5" customHeight="1">
@@ -442,11 +441,10 @@
         <x:v>説明書にURLを文字で掲載し、長いURLは折り返します。画面ではリンクとして開けます。保存画像・印刷にも同じ内容を使用します。</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>実装済み
-画面と実際の保存画像でURLの表示・折り返しを確認。印刷用の表示設定も確認。</x:v>
+        <x:v>画面・保存画像に加え、提供PDFでもURL文字列を確認済み。A4縦1ページに収まり、掲載文字の欠け・重なりはありませんでした。</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>実際の印刷プレビュー・紙面での改ページ、文字の欠け・重なりは最終確認が必要です。</x:v>
+        <x:v>今回のPDFは余白修正前のものです。修正後の再出力、および長いURLや任意入力で複数ページになる場合は追加確認が必要です。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="82.5" customHeight="1">
@@ -461,11 +459,10 @@
         <x:v>紹介状の直前に、印刷時だけ切り取り線を表示します。紹介状が次ページに移る場合も、線が紹介状側に付く設定です。通常画面と保存画像には表示しません。</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>実装済み
-通常画面・保存画像で非表示、印刷用の表示設定で表示されることを確認。</x:v>
+        <x:v>提供PDFで、説明書と紹介状の間に切り取り線があることを確認済み。通常画面・保存画像では非表示です。</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
-        <x:v>実際の印刷時に、切り取り線と紹介状が意図した位置で改ページされるかの確認が残っています。</x:v>
+        <x:v>今回のPDFは1ページです。紹介状が次ページに移る場合に切り取り線も紹介状側に付くことは、引き続き確認が必要です。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="82.5" customHeight="1">
@@ -577,8 +574,7 @@
         <x:v>紹介状から相談先の記載を削除しました。緊急度バッジも表示しません。困りごとのカテゴリ・回答内容・任意入力・作成主体「防窮研究会」は維持します。</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
-        <x:v>実装・動作確認済み
-説明書には相談先と主な困りごとのバッジがあり、紹介状にはどちらもないことを確認。</x:v>
+        <x:v>画面・保存画像に加え、提供PDFでも確認済み。説明書のみ相談先・主な困りごとのバッジがあり、紹介状にはどちらもありません。主1件＋その他3件を表示。</x:v>
       </x:c>
       <x:c r="E13" s="8" t="str">
         <x:v>主な困りごと1件・その他最大3件、その他は質問順の表示を維持。未入力の任意項目は行ごと省略します。</x:v>
@@ -616,11 +612,10 @@
 紹介状末尾：☆当紹介状は相談・支援を強制するものではありません。お困りの方が、少しでも相談や支援につながれる可能性を高めるよう準備しました。</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
-        <x:v>実装・表示確認済み
-画面と実際の保存画像で両方の注意書きを確認。</x:v>
+        <x:v>画面・保存画像に加え、提供PDFでも両方の注意書きが欠けずに表示されることを確認済み。</x:v>
       </x:c>
       <x:c r="E15" s="8" t="str">
-        <x:v>印刷にも同じ内容を使用します。印刷時の紙面全体の最終確認は残っています。</x:v>
+        <x:v>提供PDFの1ページ内での表示は確認済みです。余白修正後の再出力と、複数ページ時の配置は未確認です。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="82.5" customHeight="1">
@@ -642,10 +637,29 @@
         <x:v>更新時には途中入力のやり直しが必要です。入力した個人情報を通信やURLへ送らない構成を維持しています。</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="82.5" customHeight="1">
+      <x:c r="A17" s="9" t="str">
+        <x:v>9/26追加調整
+印刷時の左右余白</x:v>
+      </x:c>
+      <x:c r="B17" s="8" t="str">
+        <x:v>印刷用ファイルの両サイドに余白を設ける。</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="str">
+        <x:v>印刷時のみ、内容の左右にそれぞれ10mmの内側余白を追加しました。画面表示・画像保存のスタイルは変更していません。ブラウザーで指定する用紙余白とは別に確保します。</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="str">
+        <x:v>修正・ビルド済み
+余白修正はコミット0075f00に含まれます。npm ci・npm run buildは成功。パッケージ定義・ロックファイルの変更なし。</x:v>
+      </x:c>
+      <x:c r="E17" s="8" t="str">
+        <x:v>修正後の公開反映と再出力PDFは未確認です。提供済みPDFにはこの余白は含まれません。実機印刷でも枠線・文字が欠けないか確認が必要です。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd428d2959cb74f4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e25128ac73043b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>